<commit_message>
Corregir los hallazgos de la auditoría del cierre de agosto
- 1.1 Las metas Pruven emparejan productos por palabra completa
  (UTIL TOP ya no toma MANTUTIL).
- 1.2 El cumplimiento del equipo compara ventas y meta de la misma base;
  las zonas sin meta individual se informan aparte.
- 1.3 Reglas de puntaje en un solo módulo (rules.ts). Un CUMPLE del Excel
  que contradice la regla se marca Revisar o Crítico, y el simulador puede
  recalcular todo con la regla.
- 1.4 Las tarjetas de vendedor usan la hoja del vendedor y muestran la
  cifra de RESULTADOS cuando no coincide.
- 1.5 Se lee CALCULOS y se compara con las hojas y RESULTADOS.
- 1.6 Se documenta la leyenda de estados del Excel y la interpretación.
- 1.7 Los reconocimientos se verifican contra los datos (empates, ganador
  distinto; mayor incremento con el mes anterior).

Pruebas de regresión para cada punto y ejemplos con hoja CALCULOS.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/ejemplos/ejemplo-agosto-2026.xlsx
+++ b/public/ejemplos/ejemplo-agosto-2026.xlsx
@@ -9,6 +9,7 @@
     <sheet name="ZONA LLANOS" sheetId="4" r:id="rId4"/>
     <sheet name="RESULTADOS" sheetId="5" r:id="rId5"/>
     <sheet name="METAS" sheetId="6" r:id="rId6"/>
+    <sheet name="CALCULOS" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -1241,10 +1242,10 @@
         <v>2</v>
       </c>
       <c r="D6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E6">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="F6" t="str">
         <v>SI</v>
@@ -2317,4 +2318,843 @@
     <ignoredError numberStoredAsText="1" sqref="A1:J8"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H72"/>
+  <sheetData>
+    <row r="2">
+      <c r="B2" t="str">
+        <v>Pegutil</v>
+      </c>
+      <c r="C2" t="str">
+        <v>agosto</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="str">
+        <v>VENDEDOR</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Meta sacos</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Ventas</v>
+      </c>
+      <c r="E3" t="str">
+        <v>% Alcanzado</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="str">
+        <v>Laura</v>
+      </c>
+      <c r="C4">
+        <v>3500</v>
+      </c>
+      <c r="D4">
+        <v>6120</v>
+      </c>
+      <c r="E4">
+        <v>174.85714285714286</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="str">
+        <v>Mario</v>
+      </c>
+      <c r="C5">
+        <v>3500</v>
+      </c>
+      <c r="D5">
+        <v>5210</v>
+      </c>
+      <c r="E5">
+        <v>148.85714285714286</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="str">
+        <v>Patricia</v>
+      </c>
+      <c r="C6">
+        <v>2900</v>
+      </c>
+      <c r="D6">
+        <v>2632</v>
+      </c>
+      <c r="E6">
+        <v>90.75862068965517</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="str">
+        <v>Llanos</v>
+      </c>
+      <c r="C7">
+        <v>3500</v>
+      </c>
+      <c r="D7">
+        <v>2180</v>
+      </c>
+      <c r="E7">
+        <v>62.28571428571429</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="str">
+        <v>Daniela</v>
+      </c>
+      <c r="C8">
+        <v>3500</v>
+      </c>
+      <c r="D8">
+        <v>4410</v>
+      </c>
+      <c r="E8">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="C9">
+        <v>16900</v>
+      </c>
+      <c r="D9">
+        <v>20552</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="str">
+        <v>PRUVEN</v>
+      </c>
+      <c r="C11" t="str">
+        <v>agosto</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Caucho</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="str">
+        <v>VENDEDOR</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Meta caucho</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Ventas</v>
+      </c>
+      <c r="E12" t="str">
+        <v>% Alcanzado</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="str">
+        <v>Laura</v>
+      </c>
+      <c r="C13">
+        <v>700</v>
+      </c>
+      <c r="D13">
+        <v>860</v>
+      </c>
+      <c r="E13">
+        <v>122.85714285714286</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="str">
+        <v>Mario</v>
+      </c>
+      <c r="C14">
+        <v>700</v>
+      </c>
+      <c r="D14">
+        <v>640</v>
+      </c>
+      <c r="E14">
+        <v>91.42857142857143</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="str">
+        <v>Patricia</v>
+      </c>
+      <c r="C15">
+        <v>600</v>
+      </c>
+      <c r="D15">
+        <v>310</v>
+      </c>
+      <c r="E15">
+        <v>51.66666666666667</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="str">
+        <v>Llanos</v>
+      </c>
+      <c r="C16">
+        <v>700</v>
+      </c>
+      <c r="D16">
+        <v>92</v>
+      </c>
+      <c r="E16">
+        <v>13.142857142857142</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="C17">
+        <v>2700</v>
+      </c>
+      <c r="D17">
+        <v>1902</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="str">
+        <v>PRUVEN</v>
+      </c>
+      <c r="C19" t="str">
+        <v>agosto</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Mantutil</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="str">
+        <v>VENDEDOR</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Meta mantutil</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Ventas</v>
+      </c>
+      <c r="E20" t="str">
+        <v>% Alcanzado</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="str">
+        <v>Laura</v>
+      </c>
+      <c r="C21">
+        <v>100</v>
+      </c>
+      <c r="D21">
+        <v>112</v>
+      </c>
+      <c r="E21">
+        <v>112.00000000000001</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="str">
+        <v>Mario</v>
+      </c>
+      <c r="C22">
+        <v>100</v>
+      </c>
+      <c r="D22">
+        <v>104</v>
+      </c>
+      <c r="E22">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="str">
+        <v>Patricia</v>
+      </c>
+      <c r="C23">
+        <v>80</v>
+      </c>
+      <c r="D23">
+        <v>76</v>
+      </c>
+      <c r="E23">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="str">
+        <v>Llanos</v>
+      </c>
+      <c r="C24">
+        <v>80</v>
+      </c>
+      <c r="D24">
+        <v>40</v>
+      </c>
+      <c r="E24">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25">
+        <v>360</v>
+      </c>
+      <c r="D25">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="str">
+        <v>PRUVEN</v>
+      </c>
+      <c r="C27" t="str">
+        <v>agosto</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Esmalte</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="str">
+        <v>VENDEDOR</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Meta esmalte</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Ventas</v>
+      </c>
+      <c r="E28" t="str">
+        <v>% Alcanzado</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="str">
+        <v>Laura</v>
+      </c>
+      <c r="C29">
+        <v>180</v>
+      </c>
+      <c r="D29">
+        <v>214</v>
+      </c>
+      <c r="E29">
+        <v>118.88888888888889</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="str">
+        <v>Mario</v>
+      </c>
+      <c r="C30">
+        <v>120</v>
+      </c>
+      <c r="D30">
+        <v>61</v>
+      </c>
+      <c r="E30">
+        <v>50.83333333333333</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="str">
+        <v>Patricia</v>
+      </c>
+      <c r="C31">
+        <v>100</v>
+      </c>
+      <c r="D31">
+        <v>88.5</v>
+      </c>
+      <c r="E31">
+        <v>88.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="str">
+        <v>Llanos</v>
+      </c>
+      <c r="C32">
+        <v>120</v>
+      </c>
+      <c r="D32">
+        <v>33.75</v>
+      </c>
+      <c r="E32">
+        <v>28.125</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33">
+        <v>520</v>
+      </c>
+      <c r="D33">
+        <v>397.25</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="str">
+        <v>PRUVEN</v>
+      </c>
+      <c r="C35" t="str">
+        <v>agosto</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Util top</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="str">
+        <v>VENDEDOR</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Meta util top</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Ventas</v>
+      </c>
+      <c r="E36" t="str">
+        <v>% Alcanzado</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="str">
+        <v>Laura</v>
+      </c>
+      <c r="C37">
+        <v>32</v>
+      </c>
+      <c r="D37">
+        <v>71.5</v>
+      </c>
+      <c r="E37">
+        <v>223.4375</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="str">
+        <v>Mario</v>
+      </c>
+      <c r="C38">
+        <v>32</v>
+      </c>
+      <c r="D38">
+        <v>35.2</v>
+      </c>
+      <c r="E38">
+        <v>110.00000000000001</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="str">
+        <v>Patricia</v>
+      </c>
+      <c r="C39">
+        <v>32</v>
+      </c>
+      <c r="D39">
+        <v>44.1</v>
+      </c>
+      <c r="E39">
+        <v>137.8125</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="str">
+        <v>Llanos</v>
+      </c>
+      <c r="C40">
+        <v>32</v>
+      </c>
+      <c r="D40">
+        <v>6.5</v>
+      </c>
+      <c r="E40">
+        <v>20.3125</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="C41">
+        <v>128</v>
+      </c>
+      <c r="D41">
+        <v>157.3</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="str">
+        <v>PRUVEN</v>
+      </c>
+      <c r="C43" t="str">
+        <v>agosto</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Metylutil</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="str">
+        <v>VENDEDOR</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Meta metylutil</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Ventas</v>
+      </c>
+      <c r="E44" t="str">
+        <v>% Alcanzado</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="str">
+        <v>Laura</v>
+      </c>
+      <c r="C45">
+        <v>7</v>
+      </c>
+      <c r="D45">
+        <v>10</v>
+      </c>
+      <c r="E45">
+        <v>142.85714285714286</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="str">
+        <v>Mario</v>
+      </c>
+      <c r="C46">
+        <v>7</v>
+      </c>
+      <c r="D46">
+        <v>4</v>
+      </c>
+      <c r="E46">
+        <v>57.14285714285714</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="str">
+        <v>Patricia</v>
+      </c>
+      <c r="C47">
+        <v>7</v>
+      </c>
+      <c r="D47">
+        <v>8.5</v>
+      </c>
+      <c r="E47">
+        <v>121.42857142857142</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="str">
+        <v>Llanos</v>
+      </c>
+      <c r="C48">
+        <v>7</v>
+      </c>
+      <c r="D48">
+        <v>2</v>
+      </c>
+      <c r="E48">
+        <v>28.57142857142857</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="C49">
+        <v>28</v>
+      </c>
+      <c r="D49">
+        <v>24.5</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="str">
+        <v>PRUVEN</v>
+      </c>
+      <c r="C51" t="str">
+        <v>agosto</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Oxido</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="str">
+        <v>VENDEDOR</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Meta oxido</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Ventas</v>
+      </c>
+      <c r="E52" t="str">
+        <v>% Alcanzado</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" t="str">
+        <v>Laura</v>
+      </c>
+      <c r="C53">
+        <v>144</v>
+      </c>
+      <c r="D53">
+        <v>62</v>
+      </c>
+      <c r="E53">
+        <v>43.05555555555556</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="str">
+        <v>Mario</v>
+      </c>
+      <c r="C54">
+        <v>144</v>
+      </c>
+      <c r="D54">
+        <v>80</v>
+      </c>
+      <c r="E54">
+        <v>55.55555555555556</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="str">
+        <v>Patricia</v>
+      </c>
+      <c r="C55">
+        <v>144</v>
+      </c>
+      <c r="D55">
+        <v>41</v>
+      </c>
+      <c r="E55">
+        <v>28.47222222222222</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="str">
+        <v>Llanos</v>
+      </c>
+      <c r="C56">
+        <v>144</v>
+      </c>
+      <c r="D56">
+        <v>49</v>
+      </c>
+      <c r="E56">
+        <v>34.02777777777778</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57">
+        <v>576</v>
+      </c>
+      <c r="D57">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="str">
+        <v>TOTAL GALONES</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="str">
+        <v>VENDEDOR</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Meta</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Ventas</v>
+      </c>
+      <c r="E60" t="str">
+        <v>%</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="str">
+        <v>Laura</v>
+      </c>
+      <c r="C61">
+        <v>1150</v>
+      </c>
+      <c r="D61">
+        <v>1328.5</v>
+      </c>
+      <c r="E61">
+        <v>115.52173913043478</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="str">
+        <v>Mario</v>
+      </c>
+      <c r="C62">
+        <v>1000</v>
+      </c>
+      <c r="D62">
+        <v>924.2</v>
+      </c>
+      <c r="E62">
+        <v>92.42</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="str">
+        <v>Patricia</v>
+      </c>
+      <c r="C63">
+        <v>960</v>
+      </c>
+      <c r="D63">
+        <v>568.1</v>
+      </c>
+      <c r="E63">
+        <v>59.177083333333336</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" t="str">
+        <v>Llanos</v>
+      </c>
+      <c r="C64">
+        <v>1080</v>
+      </c>
+      <c r="D64">
+        <v>243.8</v>
+      </c>
+      <c r="E64">
+        <v>22.574074074074073</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" t="str">
+        <v xml:space="preserve">TOTAL GALONES </v>
+      </c>
+      <c r="C65">
+        <v>4190</v>
+      </c>
+      <c r="D65">
+        <v>3625.8</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" t="str">
+        <v>CLIENTES NUEVOS PEGUTIL</v>
+      </c>
+      <c r="F67" t="str">
+        <v>CLIENTES NUEVOS PRUVEN</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" t="str">
+        <v>VENDEDOR</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Meta</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Logrado</v>
+      </c>
+      <c r="F68" t="str">
+        <v>VENDEDOR</v>
+      </c>
+      <c r="G68" t="str">
+        <v>Meta</v>
+      </c>
+      <c r="H68" t="str">
+        <v>Logrado</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" t="str">
+        <v>Laura</v>
+      </c>
+      <c r="C69">
+        <v>2</v>
+      </c>
+      <c r="D69">
+        <v>4</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Laura</v>
+      </c>
+      <c r="G69">
+        <v>2</v>
+      </c>
+      <c r="H69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" t="str">
+        <v>Mario</v>
+      </c>
+      <c r="C70">
+        <v>2</v>
+      </c>
+      <c r="D70">
+        <v>5</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Mario</v>
+      </c>
+      <c r="G70">
+        <v>2</v>
+      </c>
+      <c r="H70">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" t="str">
+        <v>Patricia</v>
+      </c>
+      <c r="C71">
+        <v>2</v>
+      </c>
+      <c r="D71">
+        <v>5</v>
+      </c>
+      <c r="F71" t="str">
+        <v>Patricia</v>
+      </c>
+      <c r="G71">
+        <v>2</v>
+      </c>
+      <c r="H71">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="str">
+        <v>Llanos</v>
+      </c>
+      <c r="C72">
+        <v>2</v>
+      </c>
+      <c r="D72">
+        <v>1</v>
+      </c>
+      <c r="F72" t="str">
+        <v>Llanos</v>
+      </c>
+      <c r="G72">
+        <v>2</v>
+      </c>
+      <c r="H72">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H72"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>